<commit_message>
Fixed bug in InterpolationFunction, etc
</commit_message>
<xml_diff>
--- a/DataVaryingTemperature/METALSDemoMaterials.xlsx
+++ b/DataVaryingTemperature/METALSDemoMaterials.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\METALS\DataVaryingTemperature\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Krishnan Suresh\Dropbox\Personal\suresh\Software\Github\ERSL-Private\METALS\DataVaryingTemperature\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9DD09FBC-D0A5-4A20-B325-656CD0CF0A35}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{70798BB7-DC4F-42FE-AF08-CB25C04E4E97}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="1170" yWindow="1170" windowWidth="24375" windowHeight="13260" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Main" sheetId="1" r:id="rId1"/>
@@ -22,7 +22,7 @@
     <definedName name="Yield_Strength">Reference!$B$5:$D$5</definedName>
     <definedName name="Youngs_Modulus">Reference!$B$3:$D$3</definedName>
   </definedNames>
-  <calcPr calcId="0"/>
+  <calcPr calcId="0" iterateDelta="1E-4"/>
 </workbook>
 </file>
 
@@ -677,19 +677,19 @@
       <c r="F3" s="1">
         <v>77200000000</v>
       </c>
-      <c r="G3" s="1">
-        <v>193000000</v>
-      </c>
-      <c r="H3" s="1">
+      <c r="G3" s="6">
+        <v>19300000</v>
+      </c>
+      <c r="H3" s="6">
         <v>215000000</v>
       </c>
-      <c r="I3" s="1">
+      <c r="I3" s="6">
         <v>182750000</v>
       </c>
-      <c r="J3" s="1">
+      <c r="J3" s="6">
         <v>107500000</v>
       </c>
-      <c r="K3" s="1">
+      <c r="K3" s="6">
         <v>215000</v>
       </c>
       <c r="L3" s="1">
@@ -733,19 +733,19 @@
       <c r="F4" s="1">
         <v>77200000000</v>
       </c>
-      <c r="G4" s="1">
-        <v>193000000</v>
-      </c>
-      <c r="H4" s="1">
+      <c r="G4" s="6">
+        <v>19300000</v>
+      </c>
+      <c r="H4" s="6">
         <v>760000000</v>
       </c>
-      <c r="I4" s="1">
+      <c r="I4" s="6">
         <v>646000000</v>
       </c>
-      <c r="J4" s="1">
+      <c r="J4" s="6">
         <v>380000000</v>
       </c>
-      <c r="K4" s="1">
+      <c r="K4" s="6">
         <v>760000</v>
       </c>
       <c r="L4" s="1">
@@ -789,19 +789,19 @@
       <c r="F5" s="1">
         <v>80000000000</v>
       </c>
-      <c r="G5" s="1">
-        <v>200000000</v>
-      </c>
-      <c r="H5" s="1">
+      <c r="G5" s="6">
+        <v>20000000</v>
+      </c>
+      <c r="H5" s="6">
         <v>1170000000</v>
       </c>
-      <c r="I5" s="1">
+      <c r="I5" s="6">
         <v>994500000</v>
       </c>
-      <c r="J5" s="1">
+      <c r="J5" s="6">
         <v>585000000</v>
       </c>
-      <c r="K5" s="1">
+      <c r="K5" s="6">
         <v>1170000</v>
       </c>
       <c r="L5" s="1">
@@ -820,7 +820,7 @@
         <v>0.3</v>
       </c>
       <c r="Q5" s="1">
-        <v>300</v>
+        <v>350</v>
       </c>
       <c r="R5" s="1">
         <v>650000000</v>
@@ -845,19 +845,19 @@
       <c r="F6" s="1">
         <v>79600000000</v>
       </c>
-      <c r="G6" s="1">
-        <v>199000000</v>
-      </c>
-      <c r="H6" s="1">
+      <c r="G6" s="6">
+        <v>19900000</v>
+      </c>
+      <c r="H6" s="6">
         <v>550000000</v>
       </c>
-      <c r="I6" s="1">
+      <c r="I6" s="6">
         <v>467500000</v>
       </c>
-      <c r="J6" s="1">
+      <c r="J6" s="6">
         <v>275000000</v>
       </c>
-      <c r="K6" s="1">
+      <c r="K6" s="6">
         <v>550000</v>
       </c>
       <c r="L6" s="1">
@@ -901,19 +901,19 @@
       <c r="F7" s="1">
         <v>82000000000</v>
       </c>
-      <c r="G7" s="1">
-        <v>205000000</v>
-      </c>
-      <c r="H7" s="1">
+      <c r="G7" s="6">
+        <v>20500000</v>
+      </c>
+      <c r="H7" s="6">
         <v>1100000000</v>
       </c>
-      <c r="I7" s="1">
+      <c r="I7" s="6">
         <v>935000000</v>
       </c>
-      <c r="J7" s="1">
+      <c r="J7" s="6">
         <v>550000000</v>
       </c>
-      <c r="K7" s="1">
+      <c r="K7" s="6">
         <v>1100000</v>
       </c>
       <c r="L7" s="1">
@@ -957,19 +957,19 @@
       <c r="F8" s="1">
         <v>44000000000</v>
       </c>
-      <c r="G8" s="1">
-        <v>110000000</v>
-      </c>
-      <c r="H8" s="1">
+      <c r="G8" s="6">
+        <v>11000000</v>
+      </c>
+      <c r="H8" s="6">
         <v>320000000</v>
       </c>
-      <c r="I8" s="1">
+      <c r="I8" s="6">
         <v>272000000</v>
       </c>
-      <c r="J8" s="1">
+      <c r="J8" s="6">
         <v>160000000</v>
       </c>
-      <c r="K8" s="1">
+      <c r="K8" s="6">
         <v>320000</v>
       </c>
       <c r="L8" s="1">
@@ -1013,19 +1013,19 @@
       <c r="F9" s="1">
         <v>40000000000</v>
       </c>
-      <c r="G9" s="1">
-        <v>100000000</v>
-      </c>
-      <c r="H9" s="1">
+      <c r="G9" s="6">
+        <v>10000000</v>
+      </c>
+      <c r="H9" s="6">
         <v>260000000</v>
       </c>
-      <c r="I9" s="1">
+      <c r="I9" s="6">
         <v>221000000</v>
       </c>
-      <c r="J9" s="1">
+      <c r="J9" s="6">
         <v>130000000</v>
       </c>
-      <c r="K9" s="1">
+      <c r="K9" s="6">
         <v>260000</v>
       </c>
       <c r="L9" s="1">
@@ -1069,19 +1069,19 @@
       <c r="F10" s="1">
         <v>27600000000</v>
       </c>
-      <c r="G10" s="1">
-        <v>69000000</v>
-      </c>
-      <c r="H10" s="1">
+      <c r="G10" s="6">
+        <v>6900000</v>
+      </c>
+      <c r="H10" s="6">
         <v>275000000</v>
       </c>
-      <c r="I10" s="1">
+      <c r="I10" s="6">
         <v>233750000</v>
       </c>
-      <c r="J10" s="1">
+      <c r="J10" s="6">
         <v>137500000</v>
       </c>
-      <c r="K10" s="1">
+      <c r="K10" s="6">
         <v>275000</v>
       </c>
       <c r="L10" s="1">
@@ -1100,7 +1100,7 @@
         <v>0.9</v>
       </c>
       <c r="Q10" s="1">
-        <v>180</v>
+        <v>300</v>
       </c>
       <c r="R10" s="1">
         <v>100000</v>
@@ -1125,19 +1125,19 @@
       <c r="F11" s="1">
         <v>29200000000</v>
       </c>
-      <c r="G11" s="1">
-        <v>73000000</v>
-      </c>
-      <c r="H11" s="1">
+      <c r="G11" s="6">
+        <v>7300000</v>
+      </c>
+      <c r="H11" s="6">
         <v>345000000</v>
       </c>
-      <c r="I11" s="1">
+      <c r="I11" s="6">
         <v>293250000</v>
       </c>
-      <c r="J11" s="1">
+      <c r="J11" s="6">
         <v>172500000</v>
       </c>
-      <c r="K11" s="1">
+      <c r="K11" s="6">
         <v>345000</v>
       </c>
       <c r="L11" s="1">
@@ -1156,7 +1156,7 @@
         <v>0.8</v>
       </c>
       <c r="Q11" s="1">
-        <v>200</v>
+        <v>350</v>
       </c>
       <c r="R11" s="1">
         <v>100000</v>
@@ -1181,19 +1181,19 @@
       <c r="F12" s="6">
         <v>28800000000</v>
       </c>
-      <c r="G12" s="1">
-        <v>72000000</v>
-      </c>
-      <c r="H12" s="1">
+      <c r="G12" s="6">
+        <v>7200000</v>
+      </c>
+      <c r="H12" s="6">
         <v>400000000</v>
       </c>
-      <c r="I12" s="1">
+      <c r="I12" s="6">
         <v>340000000</v>
       </c>
-      <c r="J12" s="1">
+      <c r="J12" s="6">
         <v>200000000</v>
       </c>
-      <c r="K12" s="1">
+      <c r="K12" s="6">
         <v>400000</v>
       </c>
       <c r="L12" s="1">
@@ -1212,7 +1212,7 @@
         <v>0.7</v>
       </c>
       <c r="Q12" s="1">
-        <v>200</v>
+        <v>300</v>
       </c>
       <c r="R12" s="1">
         <v>100000</v>

</xml_diff>

<commit_message>
Added temperature safety factor constraint
Commented out all the changes made in the previous
commit (capping Youngs modulus and Yield strength
, checking if they drop N orders of magnitude etc)
</commit_message>
<xml_diff>
--- a/DataVaryingTemperature/METALSDemoMaterials.xlsx
+++ b/DataVaryingTemperature/METALSDemoMaterials.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Krishnan Suresh\Dropbox\Personal\suresh\Software\Github\ERSL-Private\METALS\DataVaryingTemperature\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\METALS\DataVaryingTemperature\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{70798BB7-DC4F-42FE-AF08-CB25C04E4E97}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D3204333-AB8A-41B6-930E-4BDA5DC439AF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1170" yWindow="1170" windowWidth="24375" windowHeight="13260" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Main" sheetId="1" r:id="rId1"/>
@@ -708,7 +708,7 @@
         <v>0.5</v>
       </c>
       <c r="Q3" s="1">
-        <v>900</v>
+        <v>1200</v>
       </c>
       <c r="R3" s="1">
         <v>500000000</v>
@@ -764,7 +764,7 @@
         <v>0.4</v>
       </c>
       <c r="Q4" s="1">
-        <v>800</v>
+        <v>1200</v>
       </c>
       <c r="R4" s="1">
         <v>550000000</v>

</xml_diff>

<commit_message>
DemoMaterials Result for LBracket
</commit_message>
<xml_diff>
--- a/DataVaryingTemperature/METALSDemoMaterials.xlsx
+++ b/DataVaryingTemperature/METALSDemoMaterials.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\METALS\DataVaryingTemperature\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Dropbox\Personal\suresh\Software\Github\ERSL-Private\METALS\DataVaryingTemperature\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D3204333-AB8A-41B6-930E-4BDA5DC439AF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FC9A8D3B-8423-4D42-8965-A0A45E1234D4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Main" sheetId="1" r:id="rId1"/>
@@ -535,24 +535,24 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:R12"/>
-  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="9.109375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="20.7109375" style="1" customWidth="1"/>
+    <col min="1" max="1" width="20.6640625" style="1" customWidth="1"/>
     <col min="2" max="2" width="14" style="1" customWidth="1"/>
     <col min="3" max="3" width="11" style="1" customWidth="1"/>
-    <col min="4" max="6" width="9.28515625" style="1" customWidth="1"/>
-    <col min="7" max="7" width="12.42578125" style="1" customWidth="1"/>
-    <col min="8" max="10" width="11.7109375" style="1" customWidth="1"/>
-    <col min="11" max="14" width="10.42578125" style="1" customWidth="1"/>
+    <col min="4" max="6" width="9.33203125" style="1" customWidth="1"/>
+    <col min="7" max="7" width="12.44140625" style="1" customWidth="1"/>
+    <col min="8" max="10" width="11.6640625" style="1" customWidth="1"/>
+    <col min="11" max="14" width="10.44140625" style="1" customWidth="1"/>
     <col min="15" max="15" width="10" style="1" customWidth="1"/>
-    <col min="16" max="16" width="13.7109375" style="1" customWidth="1"/>
-    <col min="17" max="17" width="16.5703125" style="1" customWidth="1"/>
-    <col min="18" max="705" width="20.5703125" style="1" customWidth="1"/>
-    <col min="706" max="706" width="9.140625" style="1" customWidth="1"/>
-    <col min="707" max="16384" width="9.140625" style="1"/>
+    <col min="16" max="16" width="13.6640625" style="1" customWidth="1"/>
+    <col min="17" max="17" width="16.5546875" style="1" customWidth="1"/>
+    <col min="18" max="705" width="20.5546875" style="1" customWidth="1"/>
+    <col min="706" max="706" width="9.109375" style="1" customWidth="1"/>
+    <col min="707" max="16384" width="9.109375" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:18" s="2" customFormat="1" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:18" s="2" customFormat="1" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="3"/>
       <c r="B1" s="3" t="s">
         <v>0</v>
@@ -606,7 +606,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="2" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A2" s="4"/>
       <c r="B2" s="4" t="s">
         <v>17</v>
@@ -658,7 +658,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="3" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A3" s="1" t="s">
         <v>23</v>
       </c>
@@ -678,7 +678,7 @@
         <v>77200000000</v>
       </c>
       <c r="G3" s="6">
-        <v>19300000</v>
+        <v>193000000</v>
       </c>
       <c r="H3" s="6">
         <v>215000000</v>
@@ -687,10 +687,10 @@
         <v>182750000</v>
       </c>
       <c r="J3" s="6">
-        <v>107500000</v>
+        <v>10750000</v>
       </c>
       <c r="K3" s="6">
-        <v>215000</v>
+        <v>2150000</v>
       </c>
       <c r="L3" s="1">
         <v>16</v>
@@ -714,7 +714,7 @@
         <v>500000000</v>
       </c>
     </row>
-    <row r="4" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A4" s="1" t="s">
         <v>24</v>
       </c>
@@ -734,7 +734,7 @@
         <v>77200000000</v>
       </c>
       <c r="G4" s="6">
-        <v>19300000</v>
+        <v>193000000</v>
       </c>
       <c r="H4" s="6">
         <v>760000000</v>
@@ -743,10 +743,10 @@
         <v>646000000</v>
       </c>
       <c r="J4" s="6">
-        <v>380000000</v>
+        <v>38000000</v>
       </c>
       <c r="K4" s="6">
-        <v>760000</v>
+        <v>7600000</v>
       </c>
       <c r="L4" s="1">
         <v>16</v>
@@ -770,7 +770,7 @@
         <v>550000000</v>
       </c>
     </row>
-    <row r="5" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A5" s="1" t="s">
         <v>25</v>
       </c>
@@ -784,10 +784,10 @@
         <v>200000000000</v>
       </c>
       <c r="E5" s="1">
-        <v>180000000000</v>
+        <v>18000000000</v>
       </c>
       <c r="F5" s="1">
-        <v>80000000000</v>
+        <v>800000000</v>
       </c>
       <c r="G5" s="6">
         <v>20000000</v>
@@ -796,10 +796,10 @@
         <v>1170000000</v>
       </c>
       <c r="I5" s="6">
-        <v>994500000</v>
+        <v>99450000</v>
       </c>
       <c r="J5" s="6">
-        <v>585000000</v>
+        <v>58500000</v>
       </c>
       <c r="K5" s="6">
         <v>1170000</v>
@@ -826,7 +826,7 @@
         <v>650000000</v>
       </c>
     </row>
-    <row r="6" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A6" s="1" t="s">
         <v>26</v>
       </c>
@@ -840,10 +840,10 @@
         <v>199000000000</v>
       </c>
       <c r="E6" s="1">
-        <v>179100000000</v>
+        <v>17910000000</v>
       </c>
       <c r="F6" s="1">
-        <v>79600000000</v>
+        <v>796000000</v>
       </c>
       <c r="G6" s="6">
         <v>19900000</v>
@@ -852,10 +852,10 @@
         <v>550000000</v>
       </c>
       <c r="I6" s="6">
-        <v>467500000</v>
+        <v>46750000</v>
       </c>
       <c r="J6" s="6">
-        <v>275000000</v>
+        <v>27500000</v>
       </c>
       <c r="K6" s="6">
         <v>550000</v>
@@ -882,7 +882,7 @@
         <v>600000000</v>
       </c>
     </row>
-    <row r="7" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A7" s="1" t="s">
         <v>27</v>
       </c>
@@ -896,10 +896,10 @@
         <v>205000000000</v>
       </c>
       <c r="E7" s="1">
-        <v>184500000000</v>
+        <v>18450000000</v>
       </c>
       <c r="F7" s="1">
-        <v>82000000000</v>
+        <v>820000000</v>
       </c>
       <c r="G7" s="6">
         <v>20500000</v>
@@ -908,10 +908,10 @@
         <v>1100000000</v>
       </c>
       <c r="I7" s="6">
-        <v>935000000</v>
+        <v>93500000</v>
       </c>
       <c r="J7" s="6">
-        <v>550000000</v>
+        <v>55000000</v>
       </c>
       <c r="K7" s="6">
         <v>1100000</v>
@@ -938,7 +938,7 @@
         <v>600000000</v>
       </c>
     </row>
-    <row r="8" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A8" s="1" t="s">
         <v>28</v>
       </c>
@@ -955,7 +955,7 @@
         <v>99000000000</v>
       </c>
       <c r="F8" s="1">
-        <v>44000000000</v>
+        <v>440000000</v>
       </c>
       <c r="G8" s="6">
         <v>11000000</v>
@@ -964,10 +964,10 @@
         <v>320000000</v>
       </c>
       <c r="I8" s="6">
-        <v>272000000</v>
+        <v>27200000</v>
       </c>
       <c r="J8" s="6">
-        <v>160000000</v>
+        <v>16000000</v>
       </c>
       <c r="K8" s="6">
         <v>320000</v>
@@ -994,7 +994,7 @@
         <v>200000</v>
       </c>
     </row>
-    <row r="9" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A9" s="1" t="s">
         <v>29</v>
       </c>
@@ -1011,7 +1011,7 @@
         <v>90000000000</v>
       </c>
       <c r="F9" s="1">
-        <v>40000000000</v>
+        <v>400000000</v>
       </c>
       <c r="G9" s="6">
         <v>10000000</v>
@@ -1020,10 +1020,10 @@
         <v>260000000</v>
       </c>
       <c r="I9" s="6">
-        <v>221000000</v>
+        <v>22100000</v>
       </c>
       <c r="J9" s="6">
-        <v>130000000</v>
+        <v>13000000</v>
       </c>
       <c r="K9" s="6">
         <v>260000</v>
@@ -1050,7 +1050,7 @@
         <v>200000</v>
       </c>
     </row>
-    <row r="10" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A10" s="1" t="s">
         <v>30</v>
       </c>
@@ -1064,10 +1064,10 @@
         <v>69000000000</v>
       </c>
       <c r="E10" s="1">
-        <v>62100000000</v>
+        <v>2100000000</v>
       </c>
       <c r="F10" s="1">
-        <v>27600000000</v>
+        <v>276000000</v>
       </c>
       <c r="G10" s="6">
         <v>6900000</v>
@@ -1076,10 +1076,10 @@
         <v>275000000</v>
       </c>
       <c r="I10" s="6">
-        <v>233750000</v>
+        <v>23375000</v>
       </c>
       <c r="J10" s="6">
-        <v>137500000</v>
+        <v>13750000</v>
       </c>
       <c r="K10" s="6">
         <v>275000</v>
@@ -1106,7 +1106,7 @@
         <v>100000</v>
       </c>
     </row>
-    <row r="11" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A11" s="1" t="s">
         <v>31</v>
       </c>
@@ -1120,10 +1120,10 @@
         <v>73000000000</v>
       </c>
       <c r="E11" s="1">
-        <v>65700000000</v>
+        <v>6570000000</v>
       </c>
       <c r="F11" s="1">
-        <v>29200000000</v>
+        <v>292000000</v>
       </c>
       <c r="G11" s="6">
         <v>7300000</v>
@@ -1132,10 +1132,10 @@
         <v>345000000</v>
       </c>
       <c r="I11" s="6">
-        <v>293250000</v>
+        <v>29325000</v>
       </c>
       <c r="J11" s="6">
-        <v>172500000</v>
+        <v>17250000</v>
       </c>
       <c r="K11" s="6">
         <v>345000</v>
@@ -1162,7 +1162,7 @@
         <v>100000</v>
       </c>
     </row>
-    <row r="12" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A12" s="1" t="s">
         <v>32</v>
       </c>
@@ -1176,10 +1176,10 @@
         <v>72000000000</v>
       </c>
       <c r="E12" s="1">
-        <v>64800000000</v>
+        <v>6480000000</v>
       </c>
       <c r="F12" s="6">
-        <v>28800000000</v>
+        <v>288000000</v>
       </c>
       <c r="G12" s="6">
         <v>7200000</v>
@@ -1188,10 +1188,10 @@
         <v>400000000</v>
       </c>
       <c r="I12" s="6">
-        <v>340000000</v>
+        <v>34000000</v>
       </c>
       <c r="J12" s="6">
-        <v>200000000</v>
+        <v>20000000</v>
       </c>
       <c r="K12" s="6">
         <v>400000</v>
@@ -1227,12 +1227,12 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:D5"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="15.7109375" customWidth="1"/>
+    <col min="1" max="1" width="15.6640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>33</v>
       </c>
@@ -1246,7 +1246,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>0</v>
       </c>
@@ -1260,7 +1260,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>39</v>
       </c>
@@ -1274,7 +1274,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>42</v>
       </c>
@@ -1288,7 +1288,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>46</v>
       </c>

</xml_diff>